<commit_message>
Updating advanced features for bioenergy
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_advanced_features.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_advanced_features.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\SuppXLS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824B08BC-82CE-42B4-80F3-1F3B80C4BED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86AEC86-B10A-4D16-A9E4-F64B86400092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
   </bookViews>
   <sheets>
     <sheet name="veda input" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="250">
   <si>
     <t>ACT_MINLD</t>
   </si>
@@ -2765,6 +2765,9 @@
   </si>
   <si>
     <t>Nuclear P</t>
+  </si>
+  <si>
+    <t>Bio Power</t>
   </si>
 </sst>
 </file>
@@ -3248,30 +3251,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75F77616-F3F2-4CAD-9718-D78F2778A52A}">
   <dimension ref="B2:S17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.9296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.1328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.9296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8" customWidth="1"/>
-    <col min="14" max="14" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.1328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="2:19" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D2" s="2" t="s">
         <v>199</v>
       </c>
@@ -3279,7 +3282,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="2:19" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>86</v>
       </c>
@@ -3333,7 +3336,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>15</v>
       </c>
@@ -3385,7 +3388,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -3443,7 +3446,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>15</v>
       </c>
@@ -3501,7 +3504,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>22</v>
       </c>
@@ -3553,7 +3556,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>22</v>
       </c>
@@ -3611,7 +3614,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -3663,7 +3666,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="10" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>25</v>
       </c>
@@ -3721,7 +3724,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>16</v>
       </c>
@@ -3773,7 +3776,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>16</v>
       </c>
@@ -3831,7 +3834,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>13</v>
       </c>
@@ -3883,7 +3886,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>13</v>
       </c>
@@ -3942,7 +3945,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="15" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>14</v>
       </c>
@@ -3994,7 +3997,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>14</v>
       </c>
@@ -4053,7 +4056,7 @@
         <v>-aggregated*</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>5</v>
       </c>
@@ -4116,19 +4119,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA60F42B-F2D1-44E2-B5F0-15531EB389CB}">
   <dimension ref="B2:AX26"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.86328125" customWidth="1"/>
-    <col min="8" max="8" width="12.86328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.1328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="6" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="5" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="6" bestFit="1" customWidth="1"/>
@@ -4139,7 +4142,7 @@
     <col min="24" max="24" width="5" bestFit="1" customWidth="1"/>
     <col min="25" max="26" width="6" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="14.53125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="2" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="5" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="6" bestFit="1" customWidth="1"/>
@@ -4160,7 +4163,7 @@
     <col min="49" max="50" width="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:50" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="2:50" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="16" t="s">
         <v>201</v>
       </c>
@@ -4168,7 +4171,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="3" spans="2:50" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:50" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>203</v>
       </c>
@@ -4305,7 +4308,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>213</v>
       </c>
@@ -4443,7 +4446,7 @@
         <v>6.18</v>
       </c>
     </row>
-    <row r="5" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>218</v>
       </c>
@@ -4581,12 +4584,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:50" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="2:50" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="AD7" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="8" spans="2:50" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:50" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>203</v>
       </c>
@@ -4752,7 +4755,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>220</v>
       </c>
@@ -4919,7 +4922,7 @@
         <v>3.72</v>
       </c>
     </row>
-    <row r="10" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>222</v>
       </c>
@@ -5086,33 +5089,33 @@
         <v>13.27</v>
       </c>
     </row>
-    <row r="13" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B13" s="16" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="14" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
         <v>224</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="18"/>
     </row>
-    <row r="15" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B15" s="18" t="s">
         <v>225</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="18"/>
     </row>
-    <row r="16" spans="2:50" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B16" s="18" t="s">
         <v>226</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="18"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
         <v>227</v>
       </c>
@@ -5123,7 +5126,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
         <v>230</v>
       </c>
@@ -5134,7 +5137,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="20" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="2:12" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
         <v>232</v>
       </c>
@@ -5148,7 +5151,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="21" spans="2:12" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="2:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
         <v>234</v>
       </c>
@@ -5174,7 +5177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="18" t="s">
         <v>239</v>
       </c>
@@ -5201,7 +5204,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="18" t="s">
         <v>241</v>
       </c>
@@ -5225,7 +5228,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
         <v>242</v>
       </c>
@@ -5249,7 +5252,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="18" t="s">
         <v>243</v>
       </c>
@@ -5273,7 +5276,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="18" t="s">
         <v>244</v>
       </c>
@@ -5282,6 +5285,18 @@
       </c>
       <c r="D26" s="18">
         <v>135</v>
+      </c>
+      <c r="H26" t="s">
+        <v>240</v>
+      </c>
+      <c r="I26" t="s">
+        <v>249</v>
+      </c>
+      <c r="K26">
+        <v>81</v>
+      </c>
+      <c r="L26">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5293,21 +5308,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B99335-61C3-404F-89AE-B281012B672E}">
   <dimension ref="B2:K46"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.86328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.19921875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.46484375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>71</v>
       </c>
@@ -5339,7 +5354,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>15</v>
       </c>
@@ -5371,7 +5386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>15</v>
       </c>
@@ -5403,7 +5418,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -5435,7 +5450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>22</v>
       </c>
@@ -5467,7 +5482,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>22</v>
       </c>
@@ -5499,7 +5514,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>25</v>
       </c>
@@ -5531,7 +5546,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -5563,7 +5578,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>16</v>
       </c>
@@ -5595,7 +5610,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>16</v>
       </c>
@@ -5627,7 +5642,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>13</v>
       </c>
@@ -5659,7 +5674,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>13</v>
       </c>
@@ -5691,7 +5706,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>14</v>
       </c>
@@ -5723,7 +5738,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>14</v>
       </c>
@@ -5755,7 +5770,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>5</v>
       </c>
@@ -5787,12 +5802,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="17.649999999999999" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:4" ht="18" x14ac:dyDescent="0.25">
       <c r="B20" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
         <v>32</v>
       </c>
@@ -5803,7 +5818,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
         <v>35</v>
       </c>
@@ -5814,7 +5829,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="7" t="s">
         <v>38</v>
       </c>
@@ -5825,7 +5840,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="7" t="s">
         <v>41</v>
       </c>
@@ -5836,7 +5851,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="7" t="s">
         <v>44</v>
       </c>
@@ -5847,7 +5862,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="7" t="s">
         <v>47</v>
       </c>
@@ -5858,7 +5873,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="7" t="s">
         <v>50</v>
       </c>
@@ -5869,7 +5884,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="7" t="s">
         <v>53</v>
       </c>
@@ -5880,62 +5895,62 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="7" t="s">
         <v>56</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="8"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="8"/>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="8"/>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="2:2" ht="17.649999999999999" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:2" ht="18" x14ac:dyDescent="0.25">
       <c r="B40" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="8"/>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="8"/>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="8"/>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="8" t="s">
         <v>63</v>
       </c>
@@ -5952,14 +5967,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B229F05-06A6-4687-AE9F-76B22C9B7EA0}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.06640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.06640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>71</v>
       </c>
@@ -5970,7 +5985,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -5981,7 +5996,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -5992,7 +6007,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -6003,7 +6018,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -6014,7 +6029,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -6025,7 +6040,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -6036,7 +6051,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -6047,7 +6062,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -6058,7 +6073,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -6069,7 +6084,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -6080,7 +6095,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -6091,7 +6106,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -6102,7 +6117,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -6113,7 +6128,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -6132,18 +6147,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFF38888-3A6B-435C-BEC8-672A605BBC9E}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
     <col min="2" max="5" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>92</v>
       </c>
@@ -6160,7 +6175,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>97</v>
       </c>
@@ -6177,7 +6192,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>102</v>
       </c>
@@ -6194,7 +6209,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
         <v>107</v>
       </c>
@@ -6211,7 +6226,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>112</v>
       </c>
@@ -6228,7 +6243,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>117</v>
       </c>
@@ -6245,7 +6260,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>122</v>
       </c>
@@ -6262,7 +6277,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>127</v>
       </c>
@@ -6279,7 +6294,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>132</v>
       </c>
@@ -6296,7 +6311,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>137</v>
       </c>
@@ -6313,7 +6328,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>142</v>
       </c>
@@ -6330,7 +6345,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="228" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" ht="270" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>147</v>
       </c>
@@ -6347,7 +6362,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="171" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" ht="210" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>152</v>
       </c>
@@ -6364,7 +6379,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>157</v>
       </c>
@@ -6381,7 +6396,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>162</v>
       </c>
@@ -6398,7 +6413,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="171" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" ht="210" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>167</v>
       </c>
@@ -6415,7 +6430,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>172</v>
       </c>
@@ -6432,7 +6447,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>177</v>
       </c>
@@ -6449,7 +6464,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>182</v>
       </c>
@@ -6466,7 +6481,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>187</v>
       </c>
@@ -6483,7 +6498,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" ht="285" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>192</v>
       </c>
@@ -6500,7 +6515,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>197</v>
       </c>
@@ -6513,12 +6528,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01242673-D8CA-43A0-8B6A-BF87C81EBC5B}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>71</v>
       </c>
@@ -6526,7 +6541,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -6534,7 +6549,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -6542,7 +6557,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -6550,7 +6565,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -6558,7 +6573,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -6566,7 +6581,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6574,7 +6589,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Adding Bio Power instead of bioenergy to advanced features
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_advanced_features.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_advanced_features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86AEC86-B10A-4D16-A9E4-F64B86400092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C09B0B4-7116-422E-8EA0-21245B78505C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
   </bookViews>
   <sheets>
     <sheet name="veda input" sheetId="1" r:id="rId1"/>
@@ -432,9 +432,6 @@
     <t>*Size Class</t>
   </si>
   <si>
-    <t>Subcritical Coal, bioenergy</t>
-  </si>
-  <si>
     <t>Supercritical Coal, IGCC</t>
   </si>
   <si>
@@ -2768,6 +2765,9 @@
   </si>
   <si>
     <t>Bio Power</t>
+  </si>
+  <si>
+    <t>Subcritical Coal, Bio Power</t>
   </si>
 </sst>
 </file>
@@ -3258,9 +3258,9 @@
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
@@ -3268,7 +3268,7 @@
     <col min="13" max="13" width="8" customWidth="1"/>
     <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -3276,10 +3276,10 @@
   <sheetData>
     <row r="2" spans="2:19" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D2" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="2:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3314,7 +3314,7 @@
         <v>82</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M3" s="9"/>
       <c r="N3" s="3" t="s">
@@ -3854,7 +3854,7 @@
         <v>0.06</v>
       </c>
       <c r="H13" t="s">
-        <v>88</v>
+        <v>249</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>83</v>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="P13" t="str">
         <f t="shared" si="0"/>
-        <v>Subcritical Coal, bioenergy</v>
+        <v>Subcritical Coal, Bio Power</v>
       </c>
       <c r="Q13" t="str">
         <f t="shared" si="3"/>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="H14" t="str">
         <f>H13</f>
-        <v>Subcritical Coal, bioenergy</v>
+        <v>Subcritical Coal, Bio Power</v>
       </c>
       <c r="I14" t="s">
         <v>76</v>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="P14" t="str">
         <f t="shared" si="0"/>
-        <v>Subcritical Coal, bioenergy</v>
+        <v>Subcritical Coal, Bio Power</v>
       </c>
       <c r="Q14" t="str">
         <f t="shared" si="3"/>
@@ -3965,7 +3965,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="H15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>83</v>
@@ -4076,7 +4076,7 @@
         <v>0.1</v>
       </c>
       <c r="H17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>83</v>
@@ -4165,39 +4165,39 @@
   <sheetData>
     <row r="2" spans="2:50" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="AD2" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="3" spans="2:50" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" t="s">
         <v>203</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>204</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>205</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>206</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>207</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>208</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>209</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>210</v>
-      </c>
-      <c r="J3" t="s">
-        <v>211</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -4245,7 +4245,7 @@
         <v>200</v>
       </c>
       <c r="AD3" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AE3" s="3">
         <f t="shared" ref="AE3:AS4" si="0">K3</f>
@@ -4310,25 +4310,25 @@
     </row>
     <row r="4" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" t="s">
         <v>213</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>214</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F4" t="s">
         <v>215</v>
-      </c>
-      <c r="E4" t="s">
-        <v>215</v>
-      </c>
-      <c r="F4" t="s">
-        <v>216</v>
       </c>
       <c r="G4" s="17">
         <v>39.18</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I4" s="17">
         <v>43.5</v>
@@ -4448,25 +4448,25 @@
     </row>
     <row r="5" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C5" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" t="s">
         <v>218</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F5" t="s">
         <v>215</v>
-      </c>
-      <c r="D5" t="s">
-        <v>219</v>
-      </c>
-      <c r="E5" t="s">
-        <v>215</v>
-      </c>
-      <c r="F5" t="s">
-        <v>216</v>
       </c>
       <c r="G5" s="17">
         <v>19.34</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I5" s="17">
         <v>28.67</v>
@@ -4586,30 +4586,30 @@
     </row>
     <row r="7" spans="2:50" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="AD7" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="2:50" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" t="s">
         <v>203</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>204</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>205</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>206</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>207</v>
       </c>
-      <c r="G8" t="s">
-        <v>208</v>
-      </c>
       <c r="H8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -4672,7 +4672,7 @@
         <v>200</v>
       </c>
       <c r="AD8" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AE8" s="3">
         <f t="shared" ref="AE8:AT10" si="2">I8</f>
@@ -4757,19 +4757,19 @@
     </row>
     <row r="9" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
+        <v>219</v>
+      </c>
+      <c r="C9" t="s">
+        <v>214</v>
+      </c>
+      <c r="D9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" t="s">
+        <v>214</v>
+      </c>
+      <c r="F9" t="s">
         <v>220</v>
-      </c>
-      <c r="C9" t="s">
-        <v>215</v>
-      </c>
-      <c r="D9" t="s">
-        <v>215</v>
-      </c>
-      <c r="E9" t="s">
-        <v>215</v>
-      </c>
-      <c r="F9" t="s">
-        <v>221</v>
       </c>
       <c r="G9" s="17">
         <v>30.18</v>
@@ -4924,19 +4924,19 @@
     </row>
     <row r="10" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G10" s="17">
         <v>19.73</v>
@@ -5091,47 +5091,47 @@
     </row>
     <row r="13" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B13" s="16" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="18"/>
     </row>
     <row r="15" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B15" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="18"/>
     </row>
     <row r="16" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B16" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="18"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="18" t="s">
         <v>228</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>230</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>231</v>
       </c>
       <c r="D19" s="18">
         <v>253</v>
@@ -5139,36 +5139,36 @@
     </row>
     <row r="20" spans="2:12" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D20" s="18">
         <v>203</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21" spans="2:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>234</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>235</v>
       </c>
       <c r="D21" s="18">
         <v>82</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="J21" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="K21" s="3">
         <v>2019</v>
@@ -5179,22 +5179,22 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D22" s="18">
         <v>242</v>
       </c>
       <c r="H22" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I22" t="s">
+        <v>245</v>
+      </c>
+      <c r="J22" t="s">
         <v>246</v>
-      </c>
-      <c r="J22" t="s">
-        <v>247</v>
       </c>
       <c r="K22">
         <f>AD4</f>
@@ -5206,16 +5206,16 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D23" s="18">
         <v>226</v>
       </c>
       <c r="H23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I23" t="s">
         <v>80</v>
@@ -5230,16 +5230,16 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D24" s="18">
         <v>174</v>
       </c>
       <c r="H24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
@@ -5254,16 +5254,16 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="18" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D25" s="18">
         <v>258</v>
       </c>
       <c r="H25" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I25" t="s">
         <v>15</v>
@@ -5278,19 +5278,19 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="C26" s="18" t="s">
         <v>244</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>245</v>
       </c>
       <c r="D26" s="18">
         <v>135</v>
       </c>
       <c r="H26" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I26" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K26">
         <v>81</v>
@@ -5982,7 +5982,7 @@
         <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -6155,369 +6155,369 @@
   <sheetData>
     <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="C3" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="D3" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>95</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="E4" s="14" t="s">
         <v>100</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="E5" s="14" t="s">
         <v>105</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="E6" s="14" t="s">
         <v>110</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="E7" s="14" t="s">
         <v>115</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="E8" s="14" t="s">
         <v>120</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="E9" s="14" t="s">
         <v>125</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="E10" s="14" t="s">
         <v>130</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="E11" s="14" t="s">
         <v>135</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="D12" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="E12" s="14" t="s">
         <v>140</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="E13" s="14" t="s">
         <v>145</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="270" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="C14" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="E14" s="14" t="s">
         <v>150</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="210" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="C15" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="D15" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="E15" s="14" t="s">
         <v>155</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="C16" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="E16" s="14" t="s">
         <v>160</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>165</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="210" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="D18" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="E18" s="14" t="s">
         <v>170</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="C19" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="D19" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="E19" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="C20" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="E20" s="14" t="s">
         <v>180</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="B21" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="C21" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="D21" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="E21" s="14" t="s">
         <v>185</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B22" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="C22" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="D22" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="E22" s="14" t="s">
         <v>190</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="285" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="C23" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="D23" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="E23" s="14" t="s">
         <v>195</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removing act_time, act_ups and act_cstup from advanced features
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_advanced_features.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_advanced_features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C09B0B4-7116-422E-8EA0-21245B78505C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41ADF66B-9E92-406D-AA83-F1DBA7B5E5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
   </bookViews>
   <sheets>
     <sheet name="veda input" sheetId="1" r:id="rId1"/>
@@ -435,9 +435,6 @@
     <t>Supercritical Coal, IGCC</t>
   </si>
   <si>
-    <t>~TFM_INS-AT: limtype=LO</t>
-  </si>
-  <si>
     <t>Decommissioning Cost Estimates for Thermal Power Technologies (in 2023 USD)</t>
   </si>
   <si>
@@ -2716,9 +2713,6 @@
     <t xml:space="preserve">Coal Steam 40 </t>
   </si>
   <si>
-    <t>~TFM_INS-TS</t>
-  </si>
-  <si>
     <t xml:space="preserve">Combined Cycle 30 </t>
   </si>
   <si>
@@ -2768,12 +2762,21 @@
   </si>
   <si>
     <t>Subcritical Coal, Bio Power</t>
+  </si>
+  <si>
+    <t>TFM_INS-TS</t>
+  </si>
+  <si>
+    <t>TFM_INS-AT: limtype=LO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0"/>
+  </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2893,7 +2896,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
@@ -2933,6 +2936,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="3"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Good" xfId="3" builtinId="26"/>
@@ -3250,36 +3254,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75F77616-F3F2-4CAD-9718-D78F2778A52A}">
-  <dimension ref="B2:S17"/>
+  <dimension ref="B2:S61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8" customWidth="1"/>
     <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D2" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>89</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="2:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3293,28 +3297,19 @@
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>3</v>
+        <v>74</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>4</v>
+        <v>82</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M3" s="9"/>
       <c r="N3" s="3" t="s">
@@ -3346,22 +3341,13 @@
       <c r="D4">
         <v>0.35000000000000003</v>
       </c>
-      <c r="E4">
-        <v>1.5</v>
-      </c>
-      <c r="F4">
-        <v>0.8</v>
-      </c>
-      <c r="G4">
-        <v>0.02</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="E4" t="s">
         <v>15</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L4" s="1">
+      <c r="I4" s="1">
         <f>dcost_data!C2</f>
         <v>50</v>
       </c>
@@ -3372,19 +3358,19 @@
         <v>0.8</v>
       </c>
       <c r="P4" t="str">
-        <f t="shared" ref="P4:P17" si="0">H4</f>
+        <f>E4</f>
         <v>OCGT (Peaker)</v>
       </c>
       <c r="Q4" t="str">
-        <f>IF(I4="","",I4)</f>
+        <f>IF(F4="","",F4)</f>
         <v/>
       </c>
       <c r="R4" t="str">
-        <f t="shared" ref="R4:R17" si="1">IF(J4="","",J4)</f>
+        <f>IF(G4="","",G4)</f>
         <v/>
       </c>
       <c r="S4" t="str">
-        <f t="shared" ref="S4:S17" si="2">IF(K4="","",K4)</f>
+        <f>IF(H4="","",H4)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3398,28 +3384,19 @@
       <c r="D5">
         <v>0.3</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="E5" t="s">
         <v>15</v>
       </c>
-      <c r="I5" t="s">
+      <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="J5" t="s">
+      <c r="G5" t="s">
         <v>77</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L5" s="1">
+      <c r="I5" s="1">
         <f>dcost_data!C3</f>
         <v>40</v>
       </c>
@@ -3430,19 +3407,19 @@
         <v>1</v>
       </c>
       <c r="P5" t="str">
-        <f t="shared" si="0"/>
+        <f>E5</f>
         <v>OCGT (Peaker)</v>
       </c>
       <c r="Q5" t="str">
-        <f t="shared" ref="Q5:Q17" si="3">IF(I5="","",I5)</f>
+        <f>IF(F5="","",F5)</f>
         <v>PASTI</v>
       </c>
       <c r="R5" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G5="","",G5)</f>
         <v>&lt;.2</v>
       </c>
       <c r="S5" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H5="","",H5)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3456,28 +3433,19 @@
       <c r="D6">
         <v>0.25</v>
       </c>
-      <c r="E6">
-        <v>0.5</v>
-      </c>
-      <c r="F6">
-        <v>1.2</v>
-      </c>
-      <c r="G6">
-        <v>0.01</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="E6" t="s">
         <v>15</v>
       </c>
-      <c r="I6" t="s">
+      <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="J6" t="s">
+      <c r="G6" t="s">
         <v>85</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L6" s="1">
+      <c r="I6" s="1">
         <f>dcost_data!C4</f>
         <v>30</v>
       </c>
@@ -3488,19 +3456,19 @@
         <v>1.2</v>
       </c>
       <c r="P6" t="str">
-        <f t="shared" si="0"/>
+        <f>E6</f>
         <v>OCGT (Peaker)</v>
       </c>
       <c r="Q6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F6="","",F6)</f>
         <v>PASTI</v>
       </c>
       <c r="R6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G6="","",G6)</f>
         <v>&lt;.05</v>
       </c>
       <c r="S6" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H6="","",H6)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3514,22 +3482,13 @@
       <c r="D7">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E7">
-        <v>4</v>
-      </c>
-      <c r="F7">
-        <v>0.45</v>
-      </c>
-      <c r="G7">
-        <v>0.04</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L7" s="1">
+      <c r="I7" s="1">
         <f>dcost_data!C5</f>
         <v>60</v>
       </c>
@@ -3540,19 +3499,19 @@
         <v>0.45</v>
       </c>
       <c r="P7" t="str">
-        <f t="shared" si="0"/>
+        <f>E7</f>
         <v>CCGT</v>
       </c>
       <c r="Q7" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F7="","",F7)</f>
         <v/>
       </c>
       <c r="R7" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G7="","",G7)</f>
         <v/>
       </c>
       <c r="S7" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H7="","",H7)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3566,28 +3525,19 @@
       <c r="D8">
         <v>0.5</v>
       </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8">
-        <v>0.6</v>
-      </c>
-      <c r="G8">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="E8" t="s">
         <v>22</v>
       </c>
-      <c r="I8" t="s">
+      <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="J8" t="s">
+      <c r="G8" t="s">
         <v>78</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L8" s="1">
+      <c r="I8" s="1">
         <f>dcost_data!C6</f>
         <v>50</v>
       </c>
@@ -3598,19 +3548,19 @@
         <v>0.6</v>
       </c>
       <c r="P8" t="str">
-        <f t="shared" si="0"/>
+        <f>E8</f>
         <v>CCGT</v>
       </c>
       <c r="Q8" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F8="","",F8)</f>
         <v>PASTI</v>
       </c>
       <c r="R8" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G8="","",G8)</f>
         <v>&lt;.3</v>
       </c>
       <c r="S8" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H8="","",H8)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3624,22 +3574,13 @@
       <c r="D9">
         <v>0.4</v>
       </c>
-      <c r="E9">
-        <v>5</v>
-      </c>
-      <c r="F9">
-        <v>0.3</v>
-      </c>
-      <c r="G9">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="E9" t="s">
         <v>80</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L9" s="1">
+      <c r="I9" s="1">
         <f>dcost_data!C7</f>
         <v>70</v>
       </c>
@@ -3650,19 +3591,19 @@
         <v>0.3</v>
       </c>
       <c r="P9" t="str">
-        <f t="shared" si="0"/>
+        <f>E9</f>
         <v>Gas_Oil Steam</v>
       </c>
       <c r="Q9" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F9="","",F9)</f>
         <v/>
       </c>
       <c r="R9" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G9="","",G9)</f>
         <v/>
       </c>
       <c r="S9" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H9="","",H9)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3676,28 +3617,19 @@
       <c r="D10">
         <v>0.35000000000000003</v>
       </c>
-      <c r="E10">
-        <v>3</v>
-      </c>
-      <c r="F10">
-        <v>0.4</v>
-      </c>
-      <c r="G10">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="E10" t="s">
         <v>80</v>
       </c>
-      <c r="I10" t="s">
+      <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="J10" t="s">
+      <c r="G10" t="s">
         <v>77</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L10" s="1">
+      <c r="I10" s="1">
         <f>dcost_data!C8</f>
         <v>60</v>
       </c>
@@ -3708,19 +3640,19 @@
         <v>0.4</v>
       </c>
       <c r="P10" t="str">
-        <f t="shared" si="0"/>
+        <f>E10</f>
         <v>Gas_Oil Steam</v>
       </c>
       <c r="Q10" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F10="","",F10)</f>
         <v>PASTI</v>
       </c>
       <c r="R10" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G10="","",G10)</f>
         <v>&lt;.2</v>
       </c>
       <c r="S10" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H10="","",H10)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3734,22 +3666,13 @@
       <c r="D11">
         <v>0.35000000000000003</v>
       </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
-      <c r="F11">
-        <v>0.6</v>
-      </c>
-      <c r="G11">
-        <v>0.02</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="E11" t="s">
         <v>81</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L11" s="1">
+      <c r="I11" s="1">
         <f>dcost_data!C9</f>
         <v>40</v>
       </c>
@@ -3760,19 +3683,19 @@
         <v>0.6</v>
       </c>
       <c r="P11" t="str">
-        <f t="shared" si="0"/>
+        <f>E11</f>
         <v>Int Comb</v>
       </c>
       <c r="Q11" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F11="","",F11)</f>
         <v/>
       </c>
       <c r="R11" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G11="","",G11)</f>
         <v/>
       </c>
       <c r="S11" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H11="","",H11)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3786,28 +3709,19 @@
       <c r="D12">
         <v>0.3</v>
       </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12">
-        <v>1.2</v>
-      </c>
-      <c r="G12">
-        <v>0.01</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="E12" t="s">
         <v>81</v>
       </c>
-      <c r="I12" t="s">
+      <c r="F12" t="s">
         <v>76</v>
       </c>
-      <c r="J12" t="s">
+      <c r="G12" t="s">
         <v>84</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L12" s="1">
+      <c r="I12" s="1">
         <f>dcost_data!C10</f>
         <v>30</v>
       </c>
@@ -3818,19 +3732,19 @@
         <v>1.2</v>
       </c>
       <c r="P12" t="str">
-        <f t="shared" si="0"/>
+        <f>E12</f>
         <v>Int Comb</v>
       </c>
       <c r="Q12" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F12="","",F12)</f>
         <v>PASTI</v>
       </c>
       <c r="R12" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G12="","",G12)</f>
         <v>&lt;.02</v>
       </c>
       <c r="S12" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H12="","",H12)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3844,22 +3758,13 @@
       <c r="D13">
         <v>0.42</v>
       </c>
-      <c r="E13">
-        <v>7</v>
-      </c>
-      <c r="F13">
-        <v>0.2</v>
-      </c>
-      <c r="G13">
-        <v>0.06</v>
-      </c>
-      <c r="H13" t="s">
-        <v>249</v>
-      </c>
-      <c r="K13" s="1" t="s">
+      <c r="E13" t="s">
+        <v>247</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L13" s="1">
+      <c r="I13" s="1">
         <f>dcost_data!C11</f>
         <v>100</v>
       </c>
@@ -3870,19 +3775,19 @@
         <v>0.2</v>
       </c>
       <c r="P13" t="str">
-        <f t="shared" si="0"/>
+        <f>E13</f>
         <v>Subcritical Coal, Bio Power</v>
       </c>
       <c r="Q13" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F13="","",F13)</f>
         <v/>
       </c>
       <c r="R13" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G13="","",G13)</f>
         <v/>
       </c>
       <c r="S13" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H13="","",H13)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3896,29 +3801,20 @@
       <c r="D14">
         <v>0.38</v>
       </c>
-      <c r="E14">
-        <v>5</v>
-      </c>
-      <c r="F14">
-        <v>0.3</v>
-      </c>
-      <c r="G14">
-        <v>0.04</v>
-      </c>
-      <c r="H14" t="str">
-        <f>H13</f>
+      <c r="E14" t="str">
+        <f>E13</f>
         <v>Subcritical Coal, Bio Power</v>
       </c>
-      <c r="I14" t="s">
+      <c r="F14" t="s">
         <v>76</v>
       </c>
-      <c r="J14" t="s">
+      <c r="G14" t="s">
         <v>78</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L14" s="1">
+      <c r="I14" s="1">
         <f>dcost_data!C12</f>
         <v>90</v>
       </c>
@@ -3929,19 +3825,19 @@
         <v>0.3</v>
       </c>
       <c r="P14" t="str">
-        <f t="shared" si="0"/>
+        <f>E14</f>
         <v>Subcritical Coal, Bio Power</v>
       </c>
       <c r="Q14" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F14="","",F14)</f>
         <v>PASTI</v>
       </c>
       <c r="R14" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G14="","",G14)</f>
         <v>&lt;.3</v>
       </c>
       <c r="S14" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H14="","",H14)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -3955,22 +3851,13 @@
       <c r="D15">
         <v>0.48</v>
       </c>
-      <c r="E15">
-        <v>8</v>
-      </c>
-      <c r="F15">
-        <v>0.15</v>
-      </c>
-      <c r="G15">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="E15" t="s">
         <v>88</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L15" s="1">
+      <c r="I15" s="1">
         <f>dcost_data!C13</f>
         <v>110</v>
       </c>
@@ -3981,19 +3868,19 @@
         <v>0.15</v>
       </c>
       <c r="P15" t="str">
-        <f t="shared" si="0"/>
+        <f>E15</f>
         <v>Supercritical Coal, IGCC</v>
       </c>
       <c r="Q15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F15="","",F15)</f>
         <v/>
       </c>
       <c r="R15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G15="","",G15)</f>
         <v/>
       </c>
       <c r="S15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H15="","",H15)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -4007,29 +3894,20 @@
       <c r="D16">
         <v>0.45</v>
       </c>
-      <c r="E16">
-        <v>6</v>
-      </c>
-      <c r="F16">
-        <v>0.25</v>
-      </c>
-      <c r="G16">
-        <v>0.05</v>
-      </c>
-      <c r="H16" t="str">
-        <f>H15</f>
+      <c r="E16" t="str">
+        <f>E15</f>
         <v>Supercritical Coal, IGCC</v>
       </c>
-      <c r="I16" t="s">
+      <c r="F16" t="s">
         <v>76</v>
       </c>
-      <c r="J16" t="s">
+      <c r="G16" t="s">
         <v>79</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L16" s="1">
+      <c r="I16" s="1">
         <f>dcost_data!C14</f>
         <v>100</v>
       </c>
@@ -4040,19 +3918,19 @@
         <v>0.25</v>
       </c>
       <c r="P16" t="str">
-        <f t="shared" si="0"/>
+        <f>E16</f>
         <v>Supercritical Coal, IGCC</v>
       </c>
       <c r="Q16" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F16="","",F16)</f>
         <v>PASTI</v>
       </c>
       <c r="R16" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G16="","",G16)</f>
         <v>&lt;.5</v>
       </c>
       <c r="S16" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H16="","",H16)</f>
         <v>-aggregated*</v>
       </c>
     </row>
@@ -4066,22 +3944,13 @@
       <c r="D17">
         <v>0.70000000000000007</v>
       </c>
-      <c r="E17">
-        <v>24</v>
-      </c>
-      <c r="F17">
-        <v>0.05</v>
-      </c>
-      <c r="G17">
-        <v>0.1</v>
-      </c>
-      <c r="H17" t="s">
-        <v>247</v>
-      </c>
-      <c r="K17" s="1" t="s">
+      <c r="E17" t="s">
+        <v>245</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="L17" s="1">
+      <c r="I17" s="1">
         <f>dcost_data!C15</f>
         <v>500</v>
       </c>
@@ -4092,20 +3961,185 @@
         <v>0.05</v>
       </c>
       <c r="P17" t="str">
-        <f t="shared" si="0"/>
+        <f>E17</f>
         <v>Nuclear P</v>
       </c>
       <c r="Q17" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(F17="","",F17)</f>
         <v/>
       </c>
       <c r="R17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G17="","",G17)</f>
         <v/>
       </c>
       <c r="S17" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(H17="","",H17)</f>
         <v>-aggregated*</v>
+      </c>
+    </row>
+    <row r="47" spans="5:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E47" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E48">
+        <v>1.5</v>
+      </c>
+      <c r="F48">
+        <v>0.8</v>
+      </c>
+      <c r="G48">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="49" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E50">
+        <v>0.5</v>
+      </c>
+      <c r="F50">
+        <v>1.2</v>
+      </c>
+      <c r="G50">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="51" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E51">
+        <v>4</v>
+      </c>
+      <c r="F51">
+        <v>0.45</v>
+      </c>
+      <c r="G51">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="52" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E52">
+        <v>2</v>
+      </c>
+      <c r="F52">
+        <v>0.6</v>
+      </c>
+      <c r="G52">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E53">
+        <v>5</v>
+      </c>
+      <c r="F53">
+        <v>0.3</v>
+      </c>
+      <c r="G53">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E54">
+        <v>3</v>
+      </c>
+      <c r="F54">
+        <v>0.4</v>
+      </c>
+      <c r="G54">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E55">
+        <v>2</v>
+      </c>
+      <c r="F55">
+        <v>0.6</v>
+      </c>
+      <c r="G55">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="56" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56">
+        <v>1.2</v>
+      </c>
+      <c r="G56">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="57" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E57">
+        <v>7</v>
+      </c>
+      <c r="F57" s="19">
+        <v>0.2</v>
+      </c>
+      <c r="G57">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="58" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E58">
+        <v>5</v>
+      </c>
+      <c r="F58">
+        <v>0.3</v>
+      </c>
+      <c r="G58">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="59" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E59">
+        <v>8</v>
+      </c>
+      <c r="F59">
+        <v>0.15</v>
+      </c>
+      <c r="G59">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E60">
+        <v>6</v>
+      </c>
+      <c r="F60">
+        <v>0.25</v>
+      </c>
+      <c r="G60">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="61" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E61">
+        <v>24</v>
+      </c>
+      <c r="F61">
+        <v>0.05</v>
+      </c>
+      <c r="G61">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -4165,39 +4199,39 @@
   <sheetData>
     <row r="2" spans="2:50" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="AD2" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="3" spans="2:50" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C3" t="s">
         <v>202</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>203</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>204</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>205</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>206</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>207</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>208</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>209</v>
-      </c>
-      <c r="J3" t="s">
-        <v>210</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -4245,7 +4279,7 @@
         <v>200</v>
       </c>
       <c r="AD3" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AE3" s="3">
         <f t="shared" ref="AE3:AS4" si="0">K3</f>
@@ -4310,25 +4344,25 @@
     </row>
     <row r="4" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C4" t="s">
         <v>212</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>213</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" t="s">
         <v>214</v>
-      </c>
-      <c r="E4" t="s">
-        <v>214</v>
-      </c>
-      <c r="F4" t="s">
-        <v>215</v>
       </c>
       <c r="G4" s="17">
         <v>39.18</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I4" s="17">
         <v>43.5</v>
@@ -4448,25 +4482,25 @@
     </row>
     <row r="5" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" t="s">
         <v>217</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" t="s">
         <v>214</v>
-      </c>
-      <c r="D5" t="s">
-        <v>218</v>
-      </c>
-      <c r="E5" t="s">
-        <v>214</v>
-      </c>
-      <c r="F5" t="s">
-        <v>215</v>
       </c>
       <c r="G5" s="17">
         <v>19.34</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I5" s="17">
         <v>28.67</v>
@@ -4586,30 +4620,30 @@
     </row>
     <row r="7" spans="2:50" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="AD7" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="2:50" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" t="s">
         <v>202</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>203</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>204</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>205</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>206</v>
       </c>
-      <c r="G8" t="s">
-        <v>207</v>
-      </c>
       <c r="H8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -4672,7 +4706,7 @@
         <v>200</v>
       </c>
       <c r="AD8" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AE8" s="3">
         <f t="shared" ref="AE8:AT10" si="2">I8</f>
@@ -4757,19 +4791,19 @@
     </row>
     <row r="9" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
+        <v>218</v>
+      </c>
+      <c r="C9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D9" t="s">
+        <v>213</v>
+      </c>
+      <c r="E9" t="s">
+        <v>213</v>
+      </c>
+      <c r="F9" t="s">
         <v>219</v>
-      </c>
-      <c r="C9" t="s">
-        <v>214</v>
-      </c>
-      <c r="D9" t="s">
-        <v>214</v>
-      </c>
-      <c r="E9" t="s">
-        <v>214</v>
-      </c>
-      <c r="F9" t="s">
-        <v>220</v>
       </c>
       <c r="G9" s="17">
         <v>30.18</v>
@@ -4924,19 +4958,19 @@
     </row>
     <row r="10" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G10" s="17">
         <v>19.73</v>
@@ -5091,47 +5125,47 @@
     </row>
     <row r="13" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B13" s="16" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="18"/>
     </row>
     <row r="15" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B15" s="18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="18"/>
     </row>
     <row r="16" spans="2:50" x14ac:dyDescent="0.25">
       <c r="B16" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="18"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="18" t="s">
         <v>227</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>229</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>230</v>
       </c>
       <c r="D19" s="18">
         <v>253</v>
@@ -5139,36 +5173,36 @@
     </row>
     <row r="20" spans="2:12" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D20" s="18">
         <v>203</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
     </row>
     <row r="21" spans="2:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D21" s="18">
         <v>82</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>235</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>237</v>
       </c>
       <c r="K21" s="3">
         <v>2019</v>
@@ -5179,22 +5213,22 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="18" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D22" s="18">
         <v>242</v>
       </c>
       <c r="H22" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I22" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="J22" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="K22">
         <f>AD4</f>
@@ -5206,16 +5240,16 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="18" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D23" s="18">
         <v>226</v>
       </c>
       <c r="H23" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I23" t="s">
         <v>80</v>
@@ -5230,16 +5264,16 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D24" s="18">
         <v>174</v>
       </c>
       <c r="H24" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
@@ -5254,16 +5288,16 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="18" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D25" s="18">
         <v>258</v>
       </c>
       <c r="H25" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I25" t="s">
         <v>15</v>
@@ -5278,19 +5312,19 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="18" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D26" s="18">
         <v>135</v>
       </c>
       <c r="H26" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I26" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="K26">
         <v>81</v>
@@ -5982,7 +6016,7 @@
         <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -6155,369 +6189,369 @@
   <sheetData>
     <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="C3" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="D3" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>94</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="E4" s="14" t="s">
         <v>99</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="E5" s="14" t="s">
         <v>104</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="E6" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="E7" s="14" t="s">
         <v>114</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="E8" s="14" t="s">
         <v>119</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="E9" s="14" t="s">
         <v>124</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="E10" s="14" t="s">
         <v>129</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="E11" s="14" t="s">
         <v>134</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="D12" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="E12" s="14" t="s">
         <v>139</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="E13" s="14" t="s">
         <v>144</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="270" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="C14" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="E14" s="14" t="s">
         <v>149</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="210" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="C15" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="D15" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="E15" s="14" t="s">
         <v>154</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="C16" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="E16" s="14" t="s">
         <v>159</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>164</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="210" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="D18" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="E18" s="14" t="s">
         <v>169</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="B19" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="C19" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="D19" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="E19" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="C20" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="E20" s="14" t="s">
         <v>179</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="B21" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="C21" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="D21" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="E21" s="14" t="s">
         <v>184</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="B22" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="C22" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="D22" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="E22" s="14" t="s">
         <v>189</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="285" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="C23" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="D23" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="E23" s="14" t="s">
         <v>194</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>